<commit_message>
Add new properties and components to enhance functionality
- Added `MNgay` property to multiple models with required validation and default value.
- Introduced `Id` property in several models with string length and Unicode settings.
- Updated `_Imports.razor` to include `Syncfusion.Blazor.Notifications`.
- Modified `ErrorLayout.razor` to include `<ToastComponent />`.
- Adjusted sorting in `GetAlls` methods of `ViTriFilletsController` and `LineFilletv2Controller`.
- Enhanced grid settings in various views to support dynamic page sizes.
</commit_message>
<xml_diff>
--- a/PMS/FilePrivate/RolePermistion(AutoRecovered).xlsx
+++ b/PMS/FilePrivate/RolePermistion(AutoRecovered).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\ProjectPMS\WEB PMSoft\PMS\FilePrivate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DBBE1FD-0E45-41CD-9F0E-999E4F798163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00D05576-AF66-4D84-B07B-77A504444B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="10560" windowWidth="23256" windowHeight="12456" xr2:uid="{81AC10DF-A2C0-4CB0-A2FC-C02D91FCFB17}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="1216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="1245">
   <si>
     <t>Fu</t>
   </si>
@@ -3676,6 +3676,93 @@
   </si>
   <si>
     <t>Export Vùng Nuôi / Mẫu Cá Giống Vùng Nuôi</t>
+  </si>
+  <si>
+    <t>Danh Mục HQ / Ca</t>
+  </si>
+  <si>
+    <t>Xem HQ / Ca</t>
+  </si>
+  <si>
+    <t>Thêm HQ / Ca</t>
+  </si>
+  <si>
+    <t>Sửa HQ / Ca</t>
+  </si>
+  <si>
+    <t>Xóa HQ / Ca</t>
+  </si>
+  <si>
+    <t>Import HQ / Ca</t>
+  </si>
+  <si>
+    <t>Export HQ / Ca</t>
+  </si>
+  <si>
+    <t>Danh Mục HQ / Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Xem HQ / Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Thêm HQ / Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Sửa HQ / Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Xóa HQ / Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Import HQ / Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Export HQ / Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Danh Mục HQ / Map Sản Phẩm Tính Lương</t>
+  </si>
+  <si>
+    <t>Xem HQ / Map Sản Phẩm Tính Lương</t>
+  </si>
+  <si>
+    <t>Thêm HQ / Map Sản Phẩm Tính Lương</t>
+  </si>
+  <si>
+    <t>Sửa HQ / Map Sản Phẩm Tính Lương</t>
+  </si>
+  <si>
+    <t>Xóa HQ / Map Sản Phẩm Tính Lương</t>
+  </si>
+  <si>
+    <t>Import HQ / Map Sản Phẩm Tính Lương</t>
+  </si>
+  <si>
+    <t>Export HQ / Map Sản Phẩm Tính Lương</t>
+  </si>
+  <si>
+    <t>Dashboard HQ</t>
+  </si>
+  <si>
+    <t>Xem Dashboard HQ</t>
+  </si>
+  <si>
+    <t>Báo Cáo HQ / Tổng Hợp Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Xem Báo Cáo HQ / Tổng Hợp Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Xuất Báo Cáo HQ / Tổng Hợp Nhân Viên Theo Ca</t>
+  </si>
+  <si>
+    <t>Báo Cáo HQ / Tổng Hợp Tính Lương</t>
+  </si>
+  <si>
+    <t>Xem Báo Cáo HQ / Tổng Hợp Tính Lương</t>
+  </si>
+  <si>
+    <t>Xuất Báo Cáo HQ / Tổng Hợp Tính Lương</t>
   </si>
 </sst>
 </file>
@@ -3751,11 +3838,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4071,7 +4159,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E8078CA-7F62-492A-B74A-AF85AB6DC653}">
-  <dimension ref="A1:F1035"/>
+  <dimension ref="A1:F1105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="80.7109375" customWidth="1"/>
@@ -12032,186 +12120,378 @@
       </c>
     </row>
     <row r="1013" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1013" t="s">
+      <c r="A1013" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1013" t="s">
+      <c r="B1013" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="1014" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1014" t="s">
-        <v>1162</v>
+        <v>1216</v>
       </c>
       <c r="B1014" t="s">
-        <v>1163</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="1015" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1015" t="s">
-        <v>1162</v>
+        <v>1216</v>
       </c>
       <c r="B1015" t="s">
-        <v>1164</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="1016" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1016" t="s">
-        <v>1165</v>
+        <v>1216</v>
       </c>
       <c r="B1016" t="s">
-        <v>1166</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="1017" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1017" t="s">
-        <v>1165</v>
+        <v>1216</v>
       </c>
       <c r="B1017" t="s">
-        <v>1167</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="1018" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1018" t="s">
-        <v>1168</v>
+        <v>1216</v>
       </c>
       <c r="B1018" t="s">
-        <v>1169</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="1019" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1019" t="s">
-        <v>1168</v>
+        <v>1216</v>
       </c>
       <c r="B1019" t="s">
-        <v>1170</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="1020" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1020" t="s">
-        <v>0</v>
+        <v>1223</v>
       </c>
       <c r="B1020" t="s">
-        <v>1</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="1021" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1021" t="s">
-        <v>1171</v>
+        <v>1223</v>
       </c>
       <c r="B1021" t="s">
-        <v>1172</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="1022" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1022" t="s">
-        <v>1171</v>
+        <v>1223</v>
       </c>
       <c r="B1022" t="s">
-        <v>1173</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="1023" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1023" t="s">
-        <v>1171</v>
+        <v>1223</v>
       </c>
       <c r="B1023" t="s">
-        <v>1174</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="1024" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1024" t="s">
-        <v>1171</v>
+        <v>1223</v>
       </c>
       <c r="B1024" t="s">
-        <v>1175</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="1025" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1025" t="s">
-        <v>1171</v>
+        <v>1223</v>
       </c>
       <c r="B1025" t="s">
-        <v>1176</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="1026" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1026" t="s">
-        <v>1171</v>
+        <v>1230</v>
       </c>
       <c r="B1026" t="s">
-        <v>1177</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="1027" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1027" t="s">
-        <v>1171</v>
+        <v>1230</v>
       </c>
       <c r="B1027" t="s">
-        <v>1178</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="1028" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1028" t="s">
-        <v>1171</v>
+        <v>1230</v>
       </c>
       <c r="B1028" t="s">
-        <v>1179</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="1029" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1029" t="s">
-        <v>1171</v>
+        <v>1230</v>
       </c>
       <c r="B1029" t="s">
-        <v>1180</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="1030" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1030" t="s">
-        <v>1171</v>
+        <v>1230</v>
       </c>
       <c r="B1030" t="s">
-        <v>1181</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="1031" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1031" t="s">
+        <v>1230</v>
+      </c>
+      <c r="B1031" t="s">
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="1078" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1078" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B1078" t="s">
+        <v>1238</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1079" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1079" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1080" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B1080" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1081" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B1081" t="s">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="1082" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1082" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B1082" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="1083" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1083" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B1083" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="1084" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1084" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B1084" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="1085" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1085" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B1085" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1086" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B1086" t="s">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1087" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B1087" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1088" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B1088" t="s">
+        <v>1243</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1089" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B1089" t="s">
+        <v>1244</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1090" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1090" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1091" t="s">
         <v>1171</v>
       </c>
-      <c r="B1031" t="s">
+      <c r="B1091" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1092" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1092" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1093" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1093" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1094" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1094" t="s">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1095" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1095" t="s">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1096" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1096" t="s">
+        <v>1177</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1097" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1097" t="s">
+        <v>1178</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1098" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1098" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1099" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1099" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1100" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1100" t="s">
+        <v>1181</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1101" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B1101" t="s">
         <v>1182</v>
       </c>
     </row>
-    <row r="1032" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1032" t="s">
+    <row r="1102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1102" t="s">
         <v>1171</v>
       </c>
-      <c r="B1032" t="s">
+      <c r="B1102" t="s">
         <v>1183</v>
       </c>
     </row>
-    <row r="1033" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1033" t="s">
+    <row r="1103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1103" t="s">
         <v>1171</v>
       </c>
-      <c r="B1033" t="s">
+      <c r="B1103" t="s">
         <v>1184</v>
       </c>
     </row>
-    <row r="1034" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1034" t="s">
+    <row r="1104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1104" t="s">
         <v>1171</v>
       </c>
-      <c r="B1034" t="s">
+      <c r="B1104" t="s">
         <v>1185</v>
       </c>
     </row>
-    <row r="1035" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1035" t="s">
+    <row r="1105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1105" t="s">
         <v>1171</v>
       </c>
-      <c r="B1035" t="s">
+      <c r="B1105" t="s">
         <v>1186</v>
       </c>
     </row>

</xml_diff>